<commit_message>
database updating and uploading
</commit_message>
<xml_diff>
--- a/outputs/01a01dcd-7e34-79d2-8653-af5fca58c003/Factory_OS_Feature_Change_Tracker_2026-08-20.xlsx
+++ b/outputs/01a01dcd-7e34-79d2-8653-af5fca58c003/Factory_OS_Feature_Change_Tracker_2026-08-20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diyaroongta/Downloads/factory-os/outputs/01a01dcd-7e34-79d2-8653-af5fca58c003/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE32E28-4DA5-384D-A7A8-157455452A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD479DA4-1BB8-0644-BF03-859513678678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="660" windowWidth="15200" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1840" yWindow="660" windowWidth="25740" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feature Tracker" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="268">
   <si>
     <t>FACTORY OS · FEATURE CHANGE LOG</t>
   </si>
@@ -806,6 +806,39 @@
   </si>
   <si>
     <t xml:space="preserve">Its breaking the order per line/not beign able to read it properly </t>
+  </si>
+  <si>
+    <t>1. Do part production plan -- from one whole plan put only some part of the PI in the schedule. 2. be able to edit production plan and make it manually editable - add warnings when cross boundary but give option to override</t>
+  </si>
+  <si>
+    <t>Abhay: demo of how to Add all BOMS and pictures of catalogue -- where is catalogue, where do I add images + BOM + packing list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">repair team planning/scheduling - before dispatch give option for repair -- say did any articles go for repair and how many, then create repair production plan. Add password protection to machine load -- show shortfall against which PI for all procurement </t>
+  </si>
+  <si>
+    <t xml:space="preserve">add option to give production plan for all articles on the catalogue itself - some have custom plans. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIS: check capacity utilisation + days at the bottom + add warnings for stale data, adding old Pis etc. ; add avg dispatch days. Add dispatch shoprtage percentage - order vs dispatch percentage; also show logic </t>
+  </si>
+  <si>
+    <t>L is large; rest all are small; its in ascending order. Add velcro/lace; add individual sizing from combo also</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add packing report format -- </t>
+  </si>
+  <si>
+    <t>23rd Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task for </t>
+  </si>
+  <si>
+    <t>Abhay</t>
+  </si>
+  <si>
+    <t>Diya</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1102,6 +1135,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1166,12 +1202,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FeatureChangeLog" displayName="FeatureChangeLog" ref="A7:H43" totalsRowShown="0">
-  <autoFilter ref="A7:H43" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FeatureChangeLog" displayName="FeatureChangeLog" ref="A7:H51" totalsRowShown="0">
+  <autoFilter ref="A7:H51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Change ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Tab / Area"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task for "/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Feature requested"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="What was corrected / changed"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="How it was tested"/>
@@ -1377,7 +1413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -1437,7 +1473,7 @@
     </row>
     <row r="5" spans="1:8" ht="26" customHeight="1">
       <c r="A5" s="25">
-        <f>COUNTA(A13:A106)</f>
+        <f>COUNTA(A21:A114)</f>
         <v>30</v>
       </c>
       <c r="B5" s="25"/>
@@ -1446,7 +1482,7 @@
       </c>
       <c r="D5" s="25"/>
       <c r="E5" s="26">
-        <f>MAX(B13:B106)</f>
+        <f>MAX(B21:B114)</f>
         <v>46254</v>
       </c>
       <c r="F5" s="25"/>
@@ -1463,7 +1499,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>10</v>
+        <v>265</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -1482,27 +1518,25 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="52" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="A8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
     </row>
     <row r="9" spans="1:8" ht="52" customHeight="1">
       <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3" t="s">
-        <v>256</v>
+      <c r="B9" t="s">
+        <v>264</v>
+      </c>
+      <c r="C9" t="s">
+        <v>267</v>
+      </c>
+      <c r="D9" t="s">
+        <v>258</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -1511,12 +1545,14 @@
     </row>
     <row r="10" spans="1:8" ht="52" customHeight="1">
       <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3" t="s">
-        <v>254</v>
+      <c r="B10" t="s">
+        <v>264</v>
+      </c>
+      <c r="C10" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" t="s">
+        <v>262</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -1525,12 +1561,14 @@
     </row>
     <row r="11" spans="1:8" ht="52" customHeight="1">
       <c r="A11" s="3"/>
-      <c r="B11" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3" t="s">
-        <v>253</v>
+      <c r="B11" t="s">
+        <v>264</v>
+      </c>
+      <c r="C11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D11" t="s">
+        <v>263</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -1539,12 +1577,14 @@
     </row>
     <row r="12" spans="1:8" ht="52" customHeight="1">
       <c r="A12" s="3"/>
-      <c r="B12" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3" t="s">
-        <v>252</v>
+      <c r="B12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C12" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" t="s">
+        <v>261</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -1552,794 +1592,912 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" ht="52" customHeight="1">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="3"/>
+      <c r="B13" t="s">
+        <v>264</v>
+      </c>
+      <c r="C13" t="s">
+        <v>267</v>
+      </c>
+      <c r="D13" t="s">
+        <v>259</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" ht="52" customHeight="1">
+      <c r="A14" s="3"/>
+      <c r="B14" t="s">
+        <v>264</v>
+      </c>
+      <c r="C14" t="s">
+        <v>267</v>
+      </c>
+      <c r="D14" t="s">
+        <v>260</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" ht="52" customHeight="1">
+      <c r="A15" s="3"/>
+      <c r="B15" t="s">
+        <v>264</v>
+      </c>
+      <c r="C15" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" t="s">
+        <v>257</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" ht="52" customHeight="1">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" ht="52" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" ht="52" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" ht="52" customHeight="1">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="1:8" ht="52" customHeight="1">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="1:8" ht="52" customHeight="1">
+      <c r="A21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B21" s="3">
         <v>46254</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="52" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="52" customHeight="1">
-      <c r="A15" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="5">
-        <v>46254</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="52" customHeight="1">
-      <c r="A16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="52" customHeight="1">
-      <c r="A17" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="5">
-        <v>46254</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="52" customHeight="1">
-      <c r="A18" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="52" customHeight="1">
-      <c r="A19" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="5">
-        <v>46254</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="52" customHeight="1">
-      <c r="A20" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="52" customHeight="1">
-      <c r="A21" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B21" s="5">
-        <v>46254</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="52" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>73</v>
+        <v>23</v>
       </c>
       <c r="B22" s="7">
         <v>46254</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="52" customHeight="1">
       <c r="A23" s="12" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="B23" s="5">
         <v>46254</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>82</v>
+        <v>32</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="52" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="B24" s="7">
         <v>46254</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>89</v>
+        <v>38</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="52" customHeight="1">
       <c r="A25" s="12" t="s">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="B25" s="5">
         <v>46254</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="52" customHeight="1">
       <c r="A26" s="11" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="B26" s="7">
         <v>46254</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="52" customHeight="1">
       <c r="A27" s="12" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="B27" s="5">
         <v>46254</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>106</v>
+        <v>55</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>107</v>
+        <v>56</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>108</v>
+        <v>57</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>110</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="52" customHeight="1">
       <c r="A28" s="11" t="s">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="B28" s="7">
         <v>46254</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>112</v>
+        <v>61</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>113</v>
+        <v>62</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>115</v>
+        <v>64</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>116</v>
+        <v>65</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>117</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="52" customHeight="1">
       <c r="A29" s="12" t="s">
-        <v>118</v>
+        <v>67</v>
       </c>
       <c r="B29" s="5">
         <v>46254</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>120</v>
+        <v>68</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>121</v>
+        <v>69</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>122</v>
+        <v>70</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>123</v>
+        <v>71</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>124</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="52" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>125</v>
+        <v>73</v>
       </c>
       <c r="B30" s="7">
         <v>46254</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>127</v>
+        <v>74</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>130</v>
+        <v>77</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="52" customHeight="1">
       <c r="A31" s="12" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="B31" s="5">
         <v>46254</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>136</v>
+        <v>83</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>137</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="52" customHeight="1">
       <c r="A32" s="11" t="s">
-        <v>138</v>
+        <v>85</v>
       </c>
       <c r="B32" s="7">
         <v>46254</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>139</v>
+        <v>86</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>140</v>
+        <v>87</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>141</v>
+        <v>88</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>142</v>
+        <v>89</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>143</v>
+        <v>90</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="52" customHeight="1">
       <c r="A33" s="12" t="s">
-        <v>145</v>
+        <v>92</v>
       </c>
       <c r="B33" s="5">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>119</v>
+        <v>86</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>148</v>
+        <v>95</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>149</v>
+        <v>96</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>150</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="52" customHeight="1">
       <c r="A34" s="11" t="s">
-        <v>151</v>
+        <v>98</v>
       </c>
       <c r="B34" s="7">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>152</v>
+        <v>86</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>153</v>
+        <v>99</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>154</v>
+        <v>100</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>156</v>
+        <v>102</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>157</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="52" customHeight="1">
       <c r="A35" s="12" t="s">
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="B35" s="5">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>159</v>
+        <v>106</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>160</v>
+        <v>107</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>161</v>
+        <v>108</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>162</v>
+        <v>109</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>163</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="52" customHeight="1">
       <c r="A36" s="11" t="s">
-        <v>164</v>
+        <v>111</v>
       </c>
       <c r="B36" s="7">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>165</v>
+        <v>112</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>166</v>
+        <v>113</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>167</v>
+        <v>114</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>169</v>
+        <v>116</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>170</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="26">
       <c r="A37" s="12" t="s">
-        <v>171</v>
+        <v>118</v>
       </c>
       <c r="B37" s="5">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>172</v>
+        <v>119</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>173</v>
+        <v>120</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>174</v>
+        <v>121</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>175</v>
+        <v>122</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>176</v>
+        <v>123</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="39">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="26">
       <c r="A38" s="11" t="s">
-        <v>178</v>
+        <v>125</v>
       </c>
       <c r="B38" s="7">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>179</v>
+        <v>126</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>180</v>
+        <v>127</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>181</v>
+        <v>128</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>182</v>
+        <v>129</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>183</v>
+        <v>130</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>184</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="26">
       <c r="A39" s="12" t="s">
-        <v>185</v>
+        <v>132</v>
       </c>
       <c r="B39" s="5">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>186</v>
+        <v>126</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>187</v>
+        <v>133</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>188</v>
+        <v>134</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>189</v>
+        <v>135</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>190</v>
+        <v>136</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>191</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="26">
       <c r="A40" s="11" t="s">
-        <v>192</v>
+        <v>138</v>
       </c>
       <c r="B40" s="7">
-        <v>46249</v>
+        <v>46254</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>193</v>
+        <v>140</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>194</v>
+        <v>141</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>195</v>
+        <v>142</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>196</v>
+        <v>143</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="26">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="39">
       <c r="A41" s="12" t="s">
-        <v>198</v>
+        <v>145</v>
       </c>
       <c r="B41" s="5">
         <v>46249</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="26">
+      <c r="A42" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B42" s="7">
+        <v>46249</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="26">
+      <c r="A43" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="B43" s="5">
+        <v>46249</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="39">
+      <c r="A44" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B44" s="7">
+        <v>46249</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="26">
+      <c r="A45" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="B45" s="5">
+        <v>46249</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="26">
+      <c r="A46" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="B46" s="7">
+        <v>46249</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="26">
+      <c r="A47" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="B47" s="5">
+        <v>46249</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="26">
+      <c r="A48" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="B48" s="7">
+        <v>46249</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="26">
+      <c r="A49" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="B49" s="5">
+        <v>46249</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D49" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="E49" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F49" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G49" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="H41" s="4" t="s">
+      <c r="H49" s="4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="39">
-      <c r="A42" s="13" t="s">
+    <row r="50" spans="1:8" ht="26">
+      <c r="A50" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B50" s="9">
         <v>46249</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C50" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D50" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E50" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="F42" s="8" t="s">
+      <c r="F50" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="G42" s="8" t="s">
+      <c r="G50" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="H42" s="8" t="s">
+      <c r="H50" s="8" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="34"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="36"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="36"/>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
+    <row r="51" spans="1:8">
+      <c r="A51" s="34"/>
+      <c r="B51" s="35"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="36"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2355,7 +2513,7 @@
     <mergeCell ref="G4:H4"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
-  <conditionalFormatting sqref="H13:H106">
+  <conditionalFormatting sqref="H21:H114">
     <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Working &amp; tested"/>
     <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="production check"/>
     <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Action required"/>
@@ -2364,7 +2522,7 @@
     <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Local"/>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="H13:H106" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="H21:H114" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Working &amp; tested,Implemented – production check needed,Action required,Not started"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I8:I99" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>